<commit_message>
Update to working model version from eps-maryland; needs IRA / ACC II data
</commit_message>
<xml_diff>
--- a/InputData/trans/TTLE/Transportation Technology Logit Exponents.xlsx
+++ b/InputData/trans/TTLE/Transportation Technology Logit Exponents.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25726"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaggarwal/Library/Containers/com.microsoft.Excel/Data/state-eps-data-repository/NJ/trans/TTLE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\US\Models\eps-us\InputData\trans\TTLE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C55451A0-457C-BE4B-AE76-77A65BE4D737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368BEB8D-0281-414A-9219-6B1C7CD0D9C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="9" r:id="rId1"/>
-    <sheet name="TTLE" sheetId="10" r:id="rId2"/>
+    <sheet name="A54.tranSubsector_logit_revised" sheetId="11" r:id="rId2"/>
+    <sheet name="TTLE" sheetId="10" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="67">
   <si>
     <t>ships</t>
   </si>
@@ -91,25 +92,148 @@
     <t>https://jgcri.github.io/gcam-doc/choice.html</t>
   </si>
   <si>
-    <t>Table 5 Generalized Cost Coefficient Calibration</t>
-  </si>
-  <si>
-    <t>United States EPA</t>
-  </si>
-  <si>
-    <t>Consumer Vehicle Choice Model Documentation</t>
-  </si>
-  <si>
-    <t>https://nepis.epa.gov/Exe/ZyPDF.cgi/P100EZ37.PDF?Dockey=P100EZ37.PDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">We choose a value of -3 for passenger vehicles and a value of -5 for other vehicle types, </t>
-  </si>
-  <si>
-    <t>based on the ranges in Table 5 of the cited EPA documentation.</t>
-  </si>
-  <si>
-    <t>New Jersey</t>
+    <t>Calibration</t>
+  </si>
+  <si>
+    <t>We use the value from PNNL's GCAM model across vehicle technologies.</t>
+  </si>
+  <si>
+    <t># File: A54.tranSubsector_logit_revised.csv</t>
+  </si>
+  <si>
+    <t># Title: Transportation default subsector logit exponents</t>
+  </si>
+  <si>
+    <t># Source: Documented in JIRA issue https://jira.pnnl.gov/jira/browse/JGCRI-358?src=confmacro.</t>
+  </si>
+  <si>
+    <t># Units: Unitless</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Column types: ccicc </t>
+  </si>
+  <si>
+    <t># ----------</t>
+  </si>
+  <si>
+    <t>supplysector</t>
+  </si>
+  <si>
+    <t>tranSubsector</t>
+  </si>
+  <si>
+    <t>logit.exponent</t>
+  </si>
+  <si>
+    <t>logit.factor</t>
+  </si>
+  <si>
+    <t>logit.type</t>
+  </si>
+  <si>
+    <t>trn_aviation_intl</t>
+  </si>
+  <si>
+    <t>International Aviation</t>
+  </si>
+  <si>
+    <t>absolute-cost-logit</t>
+  </si>
+  <si>
+    <t>trn_freight</t>
+  </si>
+  <si>
+    <t>Domestic Ship</t>
+  </si>
+  <si>
+    <t>Freight Rail</t>
+  </si>
+  <si>
+    <t>Fuel types and efficiency levels</t>
+  </si>
+  <si>
+    <t>trn_freight_road</t>
+  </si>
+  <si>
+    <t>Light truck</t>
+  </si>
+  <si>
+    <t>Fuel types</t>
+  </si>
+  <si>
+    <t>Medium truck</t>
+  </si>
+  <si>
+    <t>Heavy truck</t>
+  </si>
+  <si>
+    <t>trn_pass</t>
+  </si>
+  <si>
+    <t>Cycle</t>
+  </si>
+  <si>
+    <t>Domestic Aviation</t>
+  </si>
+  <si>
+    <t>HSR</t>
+  </si>
+  <si>
+    <t>Passenger Rail</t>
+  </si>
+  <si>
+    <t>Walk</t>
+  </si>
+  <si>
+    <t>trn_pass_road</t>
+  </si>
+  <si>
+    <t>Bus</t>
+  </si>
+  <si>
+    <t>trn_pass_road_LDV</t>
+  </si>
+  <si>
+    <t>2W and 3W</t>
+  </si>
+  <si>
+    <t>trn_pass_road_LDV_4W</t>
+  </si>
+  <si>
+    <t>Car</t>
+  </si>
+  <si>
+    <t>Fuel types and ICE efficiency levels</t>
+  </si>
+  <si>
+    <t>Large Car and Truck</t>
+  </si>
+  <si>
+    <t>Mini Car</t>
+  </si>
+  <si>
+    <t>trn_shipping_intl</t>
+  </si>
+  <si>
+    <t>International Ship</t>
+  </si>
+  <si>
+    <t># Passthrough tranSubsectors are listed belowabsolute-cost-logit</t>
+  </si>
+  <si>
+    <t>road</t>
+  </si>
+  <si>
+    <t>LDV</t>
+  </si>
+  <si>
+    <t>bus</t>
+  </si>
+  <si>
+    <t>4W</t>
+  </si>
+  <si>
+    <t>2W</t>
   </si>
 </sst>
 </file>
@@ -120,7 +244,7 @@
     <numFmt numFmtId="164" formatCode="###0.00_)"/>
     <numFmt numFmtId="165" formatCode="#,##0_)"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -785,22 +909,15 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="60">
     <cellStyle name="20% - Accent1" xfId="33" builtinId="30" customBuiltin="1"/>
@@ -1228,255 +1345,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C69"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:B54"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="45.5" customWidth="1"/>
+    <col min="2" max="2" width="45.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="8">
-        <v>44631</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="2" customFormat="1">
-      <c r="A4" s="1"/>
-      <c r="B4" s="7">
-        <v>2012</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" s="2" customFormat="1">
-      <c r="A5" s="1"/>
-      <c r="B5" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" s="2" customFormat="1">
-      <c r="A6" s="1"/>
-      <c r="B6" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" s="2" customFormat="1">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="2"/>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="2"/>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="B15" s="2"/>
-    </row>
-    <row r="16" spans="1:3" s="2" customFormat="1">
-      <c r="A16" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" s="2" customFormat="1">
-      <c r="A17" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" s="2" customFormat="1"/>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="2"/>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="2"/>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="B21" s="2"/>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="B22" s="2"/>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="B24" s="2"/>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="B25" s="2"/>
-    </row>
-    <row r="26" spans="1:2">
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="1:2">
-      <c r="B28" s="2"/>
-    </row>
-    <row r="29" spans="1:2">
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30" spans="1:2" s="2" customFormat="1"/>
-    <row r="31" spans="1:2" s="2" customFormat="1"/>
-    <row r="32" spans="1:2" s="2" customFormat="1"/>
-    <row r="33" spans="2:2" s="2" customFormat="1"/>
-    <row r="34" spans="2:2" s="2" customFormat="1"/>
-    <row r="35" spans="2:2" s="2" customFormat="1"/>
-    <row r="36" spans="2:2">
-      <c r="B36" s="2"/>
-    </row>
-    <row r="37" spans="2:2">
-      <c r="B37" s="2"/>
-    </row>
-    <row r="38" spans="2:2">
-      <c r="B38" s="2"/>
-    </row>
-    <row r="39" spans="2:2">
-      <c r="B39" s="2"/>
-    </row>
-    <row r="40" spans="2:2">
-      <c r="B40" s="2"/>
-    </row>
-    <row r="41" spans="2:2">
-      <c r="B41" s="2"/>
-    </row>
-    <row r="42" spans="2:2">
-      <c r="B42" s="2"/>
-    </row>
-    <row r="43" spans="2:2">
-      <c r="B43" s="2"/>
-    </row>
-    <row r="44" spans="2:2">
-      <c r="B44" s="2"/>
-    </row>
-    <row r="45" spans="2:2">
-      <c r="B45" s="2"/>
-    </row>
-    <row r="46" spans="2:2">
-      <c r="B46" s="2"/>
-    </row>
-    <row r="47" spans="2:2">
-      <c r="B47" s="2"/>
-    </row>
-    <row r="48" spans="2:2">
-      <c r="B48" s="2"/>
-    </row>
-    <row r="49" spans="1:2">
-      <c r="B49" s="2"/>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="B50" s="2"/>
-    </row>
-    <row r="51" spans="1:2">
-      <c r="B51" s="2"/>
-    </row>
-    <row r="52" spans="1:2">
-      <c r="B52" s="2"/>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="B53" s="2"/>
-    </row>
-    <row r="54" spans="1:2">
-      <c r="B54" s="2"/>
-    </row>
-    <row r="55" spans="1:2">
-      <c r="B55" s="2"/>
-    </row>
-    <row r="56" spans="1:2">
-      <c r="B56" s="2"/>
-    </row>
-    <row r="57" spans="1:2">
-      <c r="B57" s="2"/>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" s="1"/>
-      <c r="B58" s="2"/>
-    </row>
-    <row r="59" spans="1:2">
-      <c r="B59" s="2"/>
-    </row>
-    <row r="60" spans="1:2">
-      <c r="B60" s="2"/>
-    </row>
-    <row r="61" spans="1:2">
-      <c r="B61" s="2"/>
-    </row>
-    <row r="62" spans="1:2">
-      <c r="B62" s="2"/>
-    </row>
-    <row r="63" spans="1:2">
-      <c r="B63" s="2"/>
-    </row>
-    <row r="64" spans="1:2">
-      <c r="B64" s="2"/>
-    </row>
-    <row r="65" spans="2:2">
-      <c r="B65" s="2"/>
-    </row>
-    <row r="66" spans="2:2">
-      <c r="B66" s="2"/>
-    </row>
-    <row r="67" spans="2:2">
-      <c r="B67" s="2"/>
-    </row>
-    <row r="68" spans="2:2">
-      <c r="B68" s="2"/>
-    </row>
-    <row r="69" spans="2:2">
-      <c r="B69" s="2"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1485,93 +1419,524 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D97FB3F6-A063-4685-A6D1-3D6F2007ED8F}">
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8">
+        <v>-6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9">
+        <v>-6</v>
+      </c>
+      <c r="E9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10">
+        <v>-1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11">
+        <v>-8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12">
+        <v>-8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13">
+        <v>-8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14">
+        <v>-6</v>
+      </c>
+      <c r="E14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15">
+        <v>-6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16">
+        <v>-6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17">
+        <v>-1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18">
+        <v>-6</v>
+      </c>
+      <c r="E18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19">
+        <v>-3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20">
+        <v>-8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21">
+        <v>-8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22">
+        <v>-8</v>
+      </c>
+      <c r="D22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23">
+        <v>-8</v>
+      </c>
+      <c r="D23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24">
+        <v>-6</v>
+      </c>
+      <c r="E24" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26">
+        <v>-6</v>
+      </c>
+      <c r="E26" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27">
+        <v>-6</v>
+      </c>
+      <c r="E27" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28">
+        <v>-6</v>
+      </c>
+      <c r="E28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29">
+        <v>-6</v>
+      </c>
+      <c r="E29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30">
+        <v>-6</v>
+      </c>
+      <c r="E30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31">
+        <v>-6</v>
+      </c>
+      <c r="E31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="15.5" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2">
-        <v>-5</v>
-      </c>
-      <c r="C2" s="2">
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="B2">
+        <f>'A54.tranSubsector_logit_revised'!C21</f>
+        <v>-8</v>
+      </c>
+      <c r="C2">
+        <f>'A54.tranSubsector_logit_revised'!C11</f>
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4">
-        <v>-5</v>
-      </c>
-      <c r="C3" s="2">
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="B3">
+        <f>'A54.tranSubsector_logit_revised'!C19</f>
+        <v>-3</v>
+      </c>
+      <c r="C3">
+        <f>'A54.tranSubsector_logit_revised'!C13</f>
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4">
-        <v>-5</v>
-      </c>
-      <c r="C4" s="2">
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="B4">
+        <f>'A54.tranSubsector_logit_revised'!C15</f>
+        <v>-6</v>
+      </c>
+      <c r="C4">
+        <f>'A54.tranSubsector_logit_revised'!C8</f>
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="4">
-        <v>-5</v>
-      </c>
-      <c r="C5" s="2">
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="B5">
+        <f>'A54.tranSubsector_logit_revised'!C17</f>
+        <v>-1</v>
+      </c>
+      <c r="C5">
+        <f>'A54.tranSubsector_logit_revised'!C10</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="4">
-        <v>-5</v>
-      </c>
-      <c r="C6" s="2">
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="B6">
+        <f>'A54.tranSubsector_logit_revised'!C24</f>
+        <v>-6</v>
+      </c>
+      <c r="C6">
+        <f>'A54.tranSubsector_logit_revised'!C9</f>
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
-        <v>-5</v>
-      </c>
-      <c r="C7" s="2">
-        <v>-5</v>
+      <c r="B7">
+        <f>'A54.tranSubsector_logit_revised'!C20</f>
+        <v>-8</v>
+      </c>
+      <c r="C7">
+        <f>'A54.tranSubsector_logit_revised'!C20</f>
+        <v>-8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>